<commit_message>
docs: overhaul README with updated installation steps, usage commands, and documentation of new command-line arguments and status codes.
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,18 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFC00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FFC00000"/>
       <sz val="10"/>
@@ -91,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -111,7 +123,13 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -479,15 +497,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:F51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -522,16 +538,6 @@
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Singlish input types covered</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence / Rationale</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="79.95" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -546,7 +552,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>kochchara wela wenawada?</t>
+          <t>kechchara wela wenawada?</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -556,22 +562,12 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>question forms</t>
+          <t>කැච්චර වෙලා වෙනවද?</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Question forms</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The sentence is an informal question asking 'how long will it take?'. Evidence: 'kochchara' is an interrogative word (how much/many) and 'wenawada' forms the question ending — the system incorrectly splits 'kochchara' into two tokens.</t>
         </is>
       </c>
     </row>
@@ -596,20 +592,14 @@
           <t>මචං ඔය class එක කොහෙද තියෙන්නේ කියලා දන්නවාද?</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Question forms</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: An informal question about the location of a class. Evidence: 'koheda' is the Singlish question word for 'where' — the system maps it to 'කොහේද' (long ē vowel) instead of the correct short-vowel 'කොහෙද'.</t>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>මචං ඔය class එක කොහෙද තියෙන්නේ කියලා දන්නවද?</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -636,22 +626,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>කොමන්ඩ් ෆෝර්ම්ස්</t>
+          <t>මම එන්නට කලින් බලන්න</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Command forms</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: An informal command to wait until the speaker arrives. Evidence: 'balanna' is the imperative form of 'to look/wait' — the system renders the informal nasal 'kalin' as the formal 'කලින්' instead of the contracted 'කලිං'.</t>
         </is>
       </c>
     </row>
@@ -668,7 +648,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>karunakarala mata document eka email karala ewanna please</t>
+          <t>karuna karala mata document eka email karala ewanna please</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -676,20 +656,14 @@
           <t>කරුණාකරලා මට document එක email කරලා එවන්න please</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Command forms</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: A polite command to email a document. Evidence: 'karunakarala' is the compound Singlish politeness prefix — the system incorrectly splits it into two words 'කරුණා කරලා'.</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>කරුණා කරලා මට document එක email කරලා එවන්න please</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -716,22 +690,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>ග්රීටින්ග්ස්</t>
+          <t>සුබ නව වසරක් වේවා!</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Greetings</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: A traditional Sinhala New Year greeting. Evidence: 'Wewa' is the Singlish form of the benediction suffix '— වේවා' — the system maps it to 'වෙවා' (short e) instead of the correct long-vowel 'වේවා'.</t>
         </is>
       </c>
     </row>
@@ -756,20 +720,14 @@
           <t>මචං ගොඩක් කාලකොට දන්නන්, කොහොමද ඔයාලගේ බඩු?</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Greetings</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: A casual reunion greeting to a friend. Evidence: 'Machan' is an informal Singlish address term — the system drops the nasal ending, outputting 'මච' instead of 'මචං'.</t>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>මචන් ගොඩක් කලකොට දාන්නං, කොහොමද ඔයාලගෙ බඩු?</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -796,22 +754,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Requests</t>
+          <t>පොඩ්ඩක් ඔයාගේ නොබෝට් එක ගරන්න පුළුවන් ද?</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: A polite request to borrow a notebook. Evidence: 'garanna' is the Singlish infinitive for 'take/borrow' — the system drops the long ā vowel, outputting 'ගරන්න' instead of 'ගාරන්න'.</t>
         </is>
       </c>
     </row>
@@ -836,20 +784,14 @@
           <t>එයාගේ address එක මට එවන්න පුලුවන්ද, මම post කරන්න ඕනේ</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: A request for contact information to send a post. Evidence: 'ewanna' is the Singlish imperative for 'send' — the system inserts a long ē, outputting 'ඒවන්න' instead of 'එවන්න'.</t>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>එයාගේ address එක මට එවන්න පුළුවන්ද, මම පෝස්ට් කරන්න ඕනේ</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -876,22 +818,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>රෙපන්ස්</t>
+          <t>අනේ, ඒක දන්නේ නැහ්නේ</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Responses</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: An informal response expressing ignorance. Evidence: 'nehne' is a contracted Singlish tag meaning 'isn't it / don't you know' — the system expands it to 'නෙහ්නේ' instead of the contracted form 'නෑනේ'.</t>
         </is>
       </c>
     </row>
@@ -916,20 +848,14 @@
           <t>ඔහ් හරි හරි, මම ඒක බලමු, පාස්සේ කතා කරමු</t>
         </is>
       </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Responses</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: An informal response with agreement and a follow-up plan. Evidence: 'paasse' means 'later/after' — the system maps the final vowel to short e ('පාස්සෙ') instead of the long ē ('පාස්සේ').</t>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>ඔහ් හරි හරි, මම ඒක බලමු, පස්සෙ කතා කරමු</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -956,22 +882,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Repeated Words</t>
+          <t>එන්න එන්න, වෙනුඑ එක අපි</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Repeated Words</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'enna' is repeated for emphatic invitation/urging. Evidence: 'enna enna' is a Singlish pattern where repeating the imperative intensifies the call — the system drops the halant (්), outputting 'එන' instead of 'එන්න'.</t>
         </is>
       </c>
     </row>
@@ -988,28 +904,22 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>bohoma bohoma godak kashtai, heta exam thiyenawa machine learning eke</t>
+          <t xml:space="preserve"> heta exam thiyenawa machine learning eke</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>බොහොම බොහොම ගොඩක් කෂ්ටයි, හෙට exam තියෙනවා machine learning එකේ</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Repeated Words</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: 'bohoma' is repeated to intensify difficulty. Evidence: Repeating 'bohoma bohoma' is a Singlish intensifier pattern — the system maps both occurrences to the long-vowel variant 'බොහෝම' instead of 'බොහොම'.</t>
+          <t xml:space="preserve"> හෙට exam තියෙනවා machine learning එක</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>හෙට exam තියෙනවා machine learning එකේ</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1036,22 +946,12 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>ඉන්පුට්ස් with Punctuation Marks</t>
+          <t>ආහ්... මම හිතුවේ නෙහ්</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Inputs with Punctuation Marks</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The sentence opens with an interjection followed by an ellipsis. Evidence: 'ah' is a vocal interjection that maps to 'ආ' in Sinhala, and '...' indicates trailing speech — the system leaves 'ah' untransliterated.</t>
         </is>
       </c>
     </row>
@@ -1076,20 +976,14 @@
           <t>මොකක්ද?! ඔයාට ඒක කරන්න බෑ වගේ ද?!</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Inputs with Punctuation Marks</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: Uses combined '?!' punctuation for emphatic surprise. Evidence: '?!' is an informal combined punctuation mark — the system also maps 'bari' to 'බැරි' (formal) instead of the contracted informal form 'බෑ'.</t>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>මොකක්ද?! ඔයාට ඒක කරන්න බැරි වගේ ද?!</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1116,22 +1010,12 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>රෝමාණිකරණය / ස්පීලිංගේ විකෘති</t>
+          <t>මන් ඔයාට කතා කරන්න</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Romanization / Spelling Variants</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: All four words are maximally contracted with all vowels removed. Evidence: 'mn'=mang (I), 'oyt'=oyata (to you), 'kth'=katha (talk), 'krnn'=karanna (do) — the system cannot parse extreme vowel-stripped Singlish and outputs the raw input.</t>
         </is>
       </c>
     </row>
@@ -1156,20 +1040,14 @@
           <t>අපි අද restaurant එකකට ගිහිං කෑම කාමු ද මචං?</t>
         </is>
       </c>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>Romanization / Spelling Variants</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: 'mchnn' is a severely contracted spelling of 'machan' (friend). Evidence: Removing all vowels from 'machan' → 'mchnn' is a known informal Singlish contraction — the system fails to recognise it and leaves it as raw Roman text.</t>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>අපි අද restaurant එකකට ගිහින් කෑම කමු ද මචන්?</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1194,20 +1072,14 @@
           <t>මම අද project එක finish කරන්න try කරනවා</t>
         </is>
       </c>
-      <c r="E18" s="3" t="n"/>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>මම අද project එක finish කරන්න try කරනවා</t>
+        </is>
+      </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Isolated English Word Insertions in Singlish</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: Single English words 'project', 'finish', and 'try' are inserted into Singlish. Evidence: Each is a standalone English word — the system incorrectly renders 'karanna' as 'කරේනා' when it follows an English word.</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1232,20 +1104,14 @@
           <t>ඔය මගේ laptop එක charge කාරාද්ද මම වගේ කියලා?</t>
         </is>
       </c>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>Isolated English Word Insertions in Singlish</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: 'laptop' and 'charge' are isolated English insertions. Evidence: Both are standalone tech-domain English words — the system drops the long ā in 'karadda', outputting 'කරාද්ද' instead of 'කාරාද්ද'.</t>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා මගේ laptop එක charge කරද්ද මම වගේ කියලා?</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1270,20 +1136,14 @@
           <t>මම අද feeling totally drained, අපි කතා කරමු later ok?</t>
         </is>
       </c>
-      <c r="E20" s="3" t="n"/>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>මම අද feeling totally drained, අපි කතා කරමු later ඔක්?</t>
+        </is>
+      </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Multi-Word English Phrases in Singlish</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'feeling totally drained' is a consecutive three-word English phrase. Evidence: Three consecutive English words form an idiomatic phrase — the system partially distorts 'later' to 'latar' when it follows mixed Singlish.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1308,20 +1168,14 @@
           <t>මම හිතෙන්නේ office එකේ work from home rules change කරන්න ඕනේ, අද හාම දෙනෙක් work from home කරනවා වගේ, ඒකේ productivity බොහොම drop වෙලා, managers කියන්න ඕනේ in person meetings නැත්නම් progress track කරන්න බෑ, ඔයාට හරි වගේ ද අපි just get back to normal routine එක? දැං කොච්චර කාලා ගියාද?</t>
         </is>
       </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Multi-Word English Phrases in Singlish</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: Multiple multi-word English phrases — 'work from home', 'in person meetings', 'progress track', 'just get back to normal routine' — are embedded. Evidence: Each phrase consists of consecutive English words; the system fails to transliterate Singlish context around them after the first phrase.</t>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>මම හිතෙන්නේ office එකේ work from home rules change කරන්න ඕනේ, අද හම දෙන්නෙක් work from home කරනවා වගේ, ඒකේ productivity බොහොම drop වෙලා, managers කියන්න one in person meetings නැත්නම් progress track කරන්න බැරි, ඔයාට හරි වගේ ද අපි just get back to normal routine එක? දැන් කොච්චර කාලා ගියාද?</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1346,20 +1200,14 @@
           <t>ඔයාගේ phone එක software update කරන්න ඕනේ, battery drain වෙනවා වැඩි</t>
         </is>
       </c>
-      <c r="E22" s="3" t="n"/>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>ඔයාගෙ phone එක software update කරන්න ඕනේ, battery drain වෙනවා වැඩියි</t>
+        </is>
+      </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>English Digital Terms in Singlish</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'software', 'update', 'battery', and 'drain' are English digital terms. Evidence: These are technical/digital vocabulary words — the system stops transliterating the Singlish words following the first digital term.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1384,20 +1232,14 @@
           <t>server එක down නිසා work බෑ</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>English Digital Terms in Singlish</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: 'server' and 'down' are English digital terms meaning a system outage. Evidence: Both words are IT-domain digital terms — the system fails to transliterate the Singlish words surrounding them.</t>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>server එක down නිසා work බැරි</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1422,20 +1264,14 @@
           <t>Instagram එකේ reel එක දාන්නද?</t>
         </is>
       </c>
-      <c r="E24" s="3" t="n"/>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Instagram එකේ real එක දාන්නද?</t>
+        </is>
+      </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Platform/App Names in Singlish</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'Instagram' is a social-media platform name. Evidence: 'Instagram' is a proper noun for a well-known app — the system fails to transliterate the Singlish particles following the platform name.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1452,28 +1288,22 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Telegram group eke message ekak danna, Google Meet eka schedule karanna</t>
+          <t>Telegram group eke message ekaa danna, Google Meet eka schedule karanna</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Telegram group එකේ message එකක් දාන්න, Google Meet එක schedule කරන්න</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>Platform/App Names in Singlish</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: 'Telegram' and 'Google Meet' are platform/app names. Evidence: Both are proper nouns for digital communication platforms — their presence causes the system to leave all surrounding Singlish particles untransliterated.</t>
+          <t>Telegram group එකේ message එක දාන්න, Google Meet එක schedule කරන්න</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Telegram group එකේ message එක දාන්න, Google Meet එක schedule කරන්න</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1498,20 +1328,14 @@
           <t>DOB එක correct ද?</t>
         </is>
       </c>
-      <c r="E26" s="3" t="n"/>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>DOB ඒක correct ද?</t>
+        </is>
+      </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>English Abbreviations/Acronyms in Singlish</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'DOB' is the acronym for Date of Birth. Evidence: 'DOB' is an all-caps abbreviation — the system leaves both the acronym and the surrounding Singlish words ('eka', 'da') untransliterated.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1536,20 +1360,14 @@
           <t>මම POC එකක් කරන්න ඕනේ, COD payments support කරනවාද මේ site එකේ?</t>
         </is>
       </c>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>English Abbreviations/Acronyms in Singlish</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: 'POC' (Proof of Concept) and 'COD' (Cash on Delivery) are abbreviations. Evidence: Both are uppercase abbreviations embedded in Singlish — the system translates the initial Sinhala word but fails on everything after the first acronym.</t>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>මම POC එකෙක් කරන්න ඕනේ, COD payments support කරනවාද මේ site එකේ?</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1574,20 +1392,14 @@
           <t>හෙට uni එකේ exam එකක්</t>
         </is>
       </c>
-      <c r="E28" s="3" t="n"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>හෙට uni එකේ exam එකක්</t>
+        </is>
+      </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>English Clipped Forms in Singlish</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'uni' is a clipped form of 'university'. Evidence: 'uni' is a shortened English word used informally — the system keeps the Singlish particles 'eke' and 'ekak' in Roman script instead of transliterating them.</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1612,20 +1424,14 @@
           <t>gym එකේ sub කරලා හිතිය බඩු අද promo එකේ තියෙනවා</t>
         </is>
       </c>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>English Clipped Forms in Singlish</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: 'gym' is clipped from 'gymnasium' and 'promo' from 'promotion'. Evidence: Both are shortened English words embedded in Singlish — the system fails to transliterate any of the Singlish words in the sentence.</t>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>gym එකේ sub කරලා හිටිය බඩුව අද promo එකේ තියෙනවා</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1650,20 +1456,14 @@
           <t>Colombo 07 කියන්නේ කොහෙද?</t>
         </is>
       </c>
-      <c r="E30" s="3" t="n"/>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Colombo 07 කියන්නැට් කොහෙද?</t>
+        </is>
+      </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>Place Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'Colombo 07' is a Sri Lankan place name with a number. Evidence: 'Colombo 07' is a proper geographical noun — the system fails to transliterate the question words that follow the place name and number.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1688,20 +1488,14 @@
           <t>Kandy එකෙං Nuwara Eliya වලට යනවා, මෙහෙම train එකෙං</t>
         </is>
       </c>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>Place Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: 'Kandy' and 'Nuwara Eliya' are Sri Lankan city names. Evidence: Both are proper geographical nouns — the system keeps the Singlish words between the place names in Roman script, failing to transliterate them.</t>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Kandy එකෙන් Nuwara Eliya වලට යනවා, මෙහෙම train එකෙන්</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1726,20 +1520,14 @@
           <t>Nimali ගිහිංද?</t>
         </is>
       </c>
-      <c r="E32" s="3" t="n"/>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>නිමාලි ගිහින් ද?</t>
+        </is>
+      </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Person Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'Nimali' is a personal name used as the subject. Evidence: 'Nimali' is a proper noun (female personal name) — the presence of the name at the start causes the system to leave the subsequent Singlish words untransliterated.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1764,20 +1552,14 @@
           <t>Dinesh සහ Priyanka දෙන්නම project එකේ work කරනවා, සුපිරියටම</t>
         </is>
       </c>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Person Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: 'Dinesh' and 'Priyanka' are personal names. Evidence: Both are proper nouns for individuals — the system incorrectly maps 'saha' to 'sahaa' with a doubled vowel and fails on the remaining Singlish particles.</t>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Dinesh සහ Priyanka දෙන්නම project එකේ work කරනවා, සුපිරියටම</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1802,20 +1584,14 @@
           <t>මට 2nd attempt එකේ pass වෙන්නම් කියලා හිතුව</t>
         </is>
       </c>
-      <c r="E34" s="3" t="n"/>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>මට 2nd attempt එකේ pass වෙන්නම් කියලා හිතුවා</t>
+        </is>
+      </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: '2nd' contains the numeric ordinal suffix 'nd'. Evidence: '2nd' combines numeral '2' with suffix 'nd' — the system transliterates only 'මට' and then fails when it encounters the numeric-suffix token.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1840,20 +1616,14 @@
           <t>3rd floor එකේ office එක</t>
         </is>
       </c>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: '3rd' is a numeric ordinal with suffix 'rd'. Evidence: '3rd' combines the numeral '3' with the ordinal suffix 'rd' representing floor level — the system fails to transliterate the Singlish particles after this token.</t>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>3rd floor එකේ office එක</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1878,20 +1648,14 @@
           <t>USD 50 කොච්චරද රුපියෙල් වලිං?</t>
         </is>
       </c>
-      <c r="E36" s="3" t="n"/>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>USD 50 කොච්චරද රුපියල් වලින්?</t>
+        </is>
+      </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Inputs with Currency</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'USD' is a currency code for US Dollar. Evidence: 'USD' is an international currency abbreviation — the system fails to transliterate the Singlish words after the currency code and number.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1916,20 +1680,14 @@
           <t>ඒක GBP 200 විතරද, දැනිස්සිම යමු වගේ මහ ගාතියක් වගේ නේ</t>
         </is>
       </c>
-      <c r="E37" s="6" t="n"/>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>Inputs with Currency</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: 'GBP' is the currency abbreviation for British Pound Sterling. Evidence: 'GBP' is an uppercase currency code — the system fails to transliterate the surrounding Singlish words due to the mid-sentence currency code.</t>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>ඒක GBP 200 විතරද, දනිස්සම යමු වගේ මහා ගතියක් වගේ නෙහ්</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1954,20 +1712,14 @@
           <t>9:00AM අපි යනවා bus එක</t>
         </is>
       </c>
-      <c r="E38" s="3" t="n"/>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>9:00AM අපි යනවා bus එක</t>
+        </is>
+      </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Inputs with Time Formats</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: '9:00AM' is a 12-hour clock time format with AM suffix. Evidence: '9:00AM' uses a colon separator with uppercase AM — the system fails to transliterate the Singlish words that follow the time token.</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1984,28 +1736,22 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>meeting eka 2:30pm walata cancel kala, 4:00pm walata reschedule karala tiyenawa</t>
+          <t>meeting eka 2:30pm walata cancl karla, 4:00pm walata reschedule karala tiyenawa</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>meeting එක 2:30pm වලට cancel කළා, 4:00pm වලට reschedule කරලා තියෙනවා</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="n"/>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>Inputs with Time Formats</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: '2:30pm' and '4:00pm' are two time formats embedded in one sentence. Evidence: Both use lowercase pm — the system is unable to handle multiple time tokens and fails to transliterate any of the surrounding Singlish words.</t>
+          <t>meeting එක 2:30pm වලට cancel  කරලා 4:00pm වලට reschedule කරලා තියෙනවා</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>meeting එක 2:30pm වලට Cancl කරලා, 4:00pm වලට reschedule කරලා තියෙනවා</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2030,20 +1776,14 @@
           <t>March 05 birthday එක</t>
         </is>
       </c>
-      <c r="E40" s="3" t="n"/>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>මාර්තු 05 birthday එක</t>
+        </is>
+      </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>Inputs with Dates</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'March 05' is a partial date (month + day). Evidence: 'March 05' combines an English month name with a day number — the system leaves 'eka' in Roman script instead of transliterating it to 'එක'.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2060,7 +1800,7 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>2025/12/25 Christmas da, api koheda yanawa oyala?</t>
+          <t>2025/12/25 Christmas dhaa, api koheda yanawa oyala?</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -2068,20 +1808,14 @@
           <t>2025/12/25 Christmas ද, අපි කොහෙද යනවා ඔයාලා?</t>
         </is>
       </c>
-      <c r="E41" s="6" t="n"/>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>Inputs with Dates</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: '2025/12/25' is a full date in YYYY/MM/DD format with forward-slash separators. Evidence: The date format combined with the holiday name 'Christmas' causes the system to fail on all subsequent Singlish question words.</t>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>2025/12/25 Christmas දා, අපි කොහෙද යනවා ඔයාලා?</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2096,30 +1830,24 @@
           <t>M</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>500ml bottle ekak ganna, mama kaema metti karana eka widihata hadannam</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>500ml bottle එකක් ගන්න, මම කෑම මෙට්ටි කරන එක විදිහට හදන්නම්</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="n"/>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>500ml bottle ekak ganna, mama kaema box karana eka widihata hadannam</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>500ml bottle එකක් ගන්න, මම කෑම Box කරන එක විදිහට හදන්නම්</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>500ml bottle එකක් ගන්න, මම කෑම බොක්ස් කරන එක විදිහට හදන්නම්</t>
+        </is>
+      </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>Inputs with Unit of Measurements</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: '500ml' is a volume measurement unit. Evidence: '500ml' combines numeral '500' with unit abbreviation 'ml' (millilitre) — the system fails to transliterate the Singlish words that follow the unit token.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2139,25 +1867,19 @@
           <t>2kg sugar gedara genenna</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>2kg sugar ගෙදර ගෙන්න</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>2kg sugar ගෙදර ගෙනෙන්න</t>
         </is>
       </c>
-      <c r="E43" s="6" t="n"/>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>Inputs with Unit of Measurements</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: '2kg' is a mass measurement unit. Evidence: '2kg' combines numeral '2' with unit abbreviation 'kg' (kilogram) — the system fails to transliterate 'gedara genenna' into Sinhala.</t>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2182,20 +1904,14 @@
           <t>මාර එළකිරි work bro!</t>
         </is>
       </c>
-      <c r="E44" s="3" t="n"/>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>මාර එළකිරි වොක් bro!</t>
+        </is>
+      </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Inputs with Slang and Casual Phrasing</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'mara elakiri' is a Singlish slang phrase meaning 'extremely awesome'. Evidence: 'mara' is a Singlish intensifier and 'elakiri' is a slang term for 'excellent/cool' — the system fails to transliterate both slang words.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2220,20 +1936,14 @@
           <t>උඹ අයියේ, මේ project එක දාන පලයං, හාම තිස්සෙම set නේ</t>
         </is>
       </c>
-      <c r="E45" s="6" t="n"/>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>Inputs with Slang and Casual Phrasing</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: 'uba', 'palayan', and 'set neh' are casual/slang expressions. Evidence: 'uba' is a very informal second-person pronoun, 'palayan' means 'get lost' (rude dismissal), and 'set neh' means 'it's not working' in Singlish slang.</t>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>උඹ අයියෙ, මේ project එක දාන පලයන්, හම තිස්සෙම set නෙහ්</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2258,20 +1968,14 @@
           <t>මට මේ link එක එවන්න: www.example.lk, මම check කරන්න</t>
         </is>
       </c>
-      <c r="E46" s="3" t="n"/>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>මට මේ link එක එවන්න: www.example.ල්ක්, මම check කරන්න</t>
+        </is>
+      </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>Online Identifiers in Singlish</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: 'www.example.lk' is a URL (online identifier). Evidence: The web address uses 'www.' prefix — the system fails entirely when a URL is present, leaving all Singlish words in the sentence untransliterated.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2296,20 +2000,14 @@
           <t>ඔය @Kasun අය්‍යාට message කෑරාව ද, එයාට කියන්න urgent කියලා</t>
         </is>
       </c>
-      <c r="E47" s="6" t="n"/>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>Online Identifiers in Singlish</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: '@Kasun' is a social-media mention identifier. Evidence: '@Kasun' uses the '@' symbol as a social mention prefix — its presence causes the system to leave all surrounding Singlish text untransliterated.</t>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා @Kasun අයියට message කරව ද, එයාට කියන්න urgent කියලා</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2334,20 +2032,14 @@
           <t>බොහොම පිං 🙏</t>
         </is>
       </c>
-      <c r="E48" s="3" t="n"/>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>බොහොම පින් 🙏</t>
+        </is>
+      </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>Inputs Containing Emojis</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The 🙏 emoji follows Singlish text expressing gratitude. Evidence: The 🙏 emoji appears at the end of the expression 'bohoma pin' (very meritorious) — the system fails to transliterate the Singlish words when an emoji is present.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2372,20 +2064,14 @@
           <t>මචං, මෙක බලන්න 😭 අපි හදාපු වගේ නේ ඔයාගේ idea එක</t>
         </is>
       </c>
-      <c r="E49" s="6" t="n"/>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>Inputs Containing Emojis</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: The 😭 emoji is embedded mid-sentence between two Singlish clauses. Evidence: The crying emoji divides the sentence — its mid-sentence position disrupts the system's ability to transliterate any part of the input.</t>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>මචං, මේක බලන්න 😭 අපි හදපු වගේ නෙහ් ඔයාගෙ idea එක</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2410,20 +2096,14 @@
           <t>ඔය හදාපු project එක කොහෙද submit කරන්නේ කියලා දන්නවාද?</t>
         </is>
       </c>
-      <c r="E50" s="3" t="n"/>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා හදපු project එක කොහෙද submit කරන්නේ කියලා දන්නවද?</t>
+        </is>
+      </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Question forms</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: A question about where to submit a project. Evidence: 'koheda' is the question word for 'where' and 'dannawada' forms the interrogative suffix — the English word 'submit' causes the system to stop transliterating.</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2448,24 +2128,19 @@
           <t>පොඩ්ඩක් බලන්න, මම එන්න ගියාමත් දාන්න, okay ද?</t>
         </is>
       </c>
-      <c r="E51" s="6" t="n"/>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>Command forms</t>
-        </is>
-      </c>
-      <c r="H51" s="6" t="inlineStr">
-        <is>
-          <t>Rationale: Contains two imperative commands followed by a confirmation question. Evidence: 'balanna' and 'danna' are both imperative Singlish verbs — the English word 'okay' causes the system to fail on transliterating the full command sequence.</t>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>පොඩ්ඩක් බලන්න, මම එන්න ගියාමත් දාන්න, ඕකේද?</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>